<commit_message>
Baseline RAG adapter suite, parser microservices, and two-phase processing
確定スタック(OCI Enterprise AI / OCI Generative AI Cohere / Oracle 26ai)に沿って
作業ツリーに未コミットだった累積実装をベースライン化する。

- parser/chunking/retrieval/grounding/generation/guardrail/vector-index/
  evaluation/graph/agentic の各アダプターと設定 API・設定画面
- parser 層をマイクロサービス委譲へ再編(packages/rag_parser_core 共有 core +
  services/parsers/* の docling/marker/unstructured/mineru/dots_ocr 各サービス +
  backend/app/clients/parser_service の HTTP runner 注入)
- 2 段階ファイル処理(parse→人手プレビュー確認→index)と review gate
- KB 単位アダプター上書き、診断/監査/観測の拡充
- frontend 設定画面群と e2e、評価 fixtures

注: 出自は作業ツリーの累積変更。internal の health check は ruff 緑・pytest collect 正常。

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evaluation/file-processing-fixtures/budget-ja.xlsx
+++ b/evaluation/file-processing-fixtures/budget-ja.xlsx
@@ -1,3 +1,11 @@
+
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="経費" sheetId="1" r:id="rId1"/>
+  </sheets>
+</workbook>
+</file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
@@ -44,6 +52,31 @@
     <t>400円</t>
   </si>
 </sst>
+</file>
+
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="1">
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+  </fonts>
+  <fills count="1">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border/>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+  </cellXfs>
+</styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>